<commit_message>
Added location of reference device document to NFP-17.
</commit_message>
<xml_diff>
--- a/Dokumentace/Nefunkcni_pozadavky_tankovani_4.xlsx
+++ b/Dokumentace/Nefunkcni_pozadavky_tankovani_4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jirivavra/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Fueling_Management_Tool\Dokumentace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD72581-18B8-6A4A-8D63-7A56600EF5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9917A593-3E60-42BC-80C9-EF8B65ADEEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="32220" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nefunkční požadavky" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="79">
   <si>
     <t>Nefunkční požadavky</t>
   </si>
@@ -28,9 +28,6 @@
     <t>Nástroj pro správu tankování</t>
   </si>
   <si>
-    <t>Návrh k týmovému schválení. NFP-02 a NFP-07 čekají na testovací parametry; referenční zařízení pro NFP-17 dosud není určeno.</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -254,13 +251,19 @@
   </si>
   <si>
     <t>Úspěšnost rozpoznání OCR</t>
+  </si>
+  <si>
+    <t>Návrh k týmovému schválení. NFP-02 a NFP-07 čekají na testovací parametry.</t>
+  </si>
+  <si>
+    <t>Dokument s definicí referenčního zařízení.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -309,6 +312,12 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -347,11 +356,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -377,6 +387,9 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -389,11 +402,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hypertextový odkaz" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -605,13 +617,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="100" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
+    <col min="5" max="5" width="35.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -621,28 +634,28 @@
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" ht="22" customHeight="1">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
     </row>
     <row r="4" spans="1:4" ht="34" customHeight="1">
-      <c r="A4" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="A4" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1"/>
@@ -652,311 +665,314 @@
     </row>
     <row r="6" spans="1:4" ht="29" customHeight="1">
       <c r="A6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="26" customHeight="1">
+      <c r="A7" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="26" customHeight="1">
-      <c r="A7" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
     </row>
     <row r="8" spans="1:4" ht="61" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="76" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="76" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="3" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="26" customHeight="1">
+      <c r="A11" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="26" customHeight="1">
-      <c r="A11" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
     </row>
     <row r="12" spans="1:4" ht="61" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>20</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="61" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1">
       <c r="A14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="61" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="3" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="26" customHeight="1">
+      <c r="A16" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="26" customHeight="1">
-      <c r="A16" s="13" t="s">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" ht="91" customHeight="1">
+      <c r="A17" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-    </row>
-    <row r="17" spans="1:4" ht="91" customHeight="1">
-      <c r="A17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="6" t="s">
+    </row>
+    <row r="18" spans="1:5" ht="76" customHeight="1">
+      <c r="A18" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="76" customHeight="1">
-      <c r="A18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:5" ht="26" customHeight="1">
+      <c r="A19" s="9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="26" customHeight="1">
-      <c r="A19" s="13" t="s">
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+    </row>
+    <row r="20" spans="1:5" ht="61" customHeight="1">
+      <c r="A20" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-    </row>
-    <row r="20" spans="1:4" ht="61" customHeight="1">
-      <c r="A20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="C20" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="6" t="s">
+    </row>
+    <row r="21" spans="1:5" ht="76" customHeight="1">
+      <c r="A21" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="76" customHeight="1">
-      <c r="A21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="3" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="26" customHeight="1">
+      <c r="A22" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="26" customHeight="1">
-      <c r="A22" s="13" t="s">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+    </row>
+    <row r="23" spans="1:5" ht="61" customHeight="1">
+      <c r="A23" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-    </row>
-    <row r="23" spans="1:4" ht="61" customHeight="1">
-      <c r="A23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="C23" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="6" t="s">
+    </row>
+    <row r="24" spans="1:5" ht="76" customHeight="1">
+      <c r="A24" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="76" customHeight="1">
-      <c r="A24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="26" customHeight="1">
+      <c r="A25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="26" customHeight="1">
-      <c r="A25" s="13" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" ht="61" customHeight="1">
+      <c r="A26" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-    </row>
-    <row r="26" spans="1:4" ht="61" customHeight="1">
-      <c r="A26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="C26" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="6" t="s">
+    </row>
+    <row r="27" spans="1:5" ht="61" customHeight="1">
+      <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="61" customHeight="1">
-      <c r="A27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="61" customHeight="1">
+      <c r="A28" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="61" customHeight="1">
-      <c r="A28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="C28" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D28" s="6" t="s">
+    </row>
+    <row r="29" spans="1:5" ht="76" customHeight="1">
+      <c r="A29" s="4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="76" customHeight="1">
-      <c r="A29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:5">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1012,6 +1028,9 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A11:D11"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E29" r:id="rId1" xr:uid="{1B60EFB6-15CA-4EED-ADA5-9B873EEC2371}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Edit to the original file
added link to the refference device
</commit_message>
<xml_diff>
--- a/Dokumentace/Nefunkcni_pozadavky_tankovani_4.xlsx
+++ b/Dokumentace/Nefunkcni_pozadavky_tankovani_4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Fueling_Management_Tool\Dokumentace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jirivavra/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9917A593-3E60-42BC-80C9-EF8B65ADEEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DA53A6-5C79-AC4D-87FD-7E6F4F2261DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="32220" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nefunkční požadavky" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>Nefunkční požadavky</t>
   </si>
@@ -253,17 +253,14 @@
     <t>Úspěšnost rozpoznání OCR</t>
   </si>
   <si>
-    <t>Návrh k týmovému schválení. NFP-02 a NFP-07 čekají na testovací parametry.</t>
-  </si>
-  <si>
-    <t>Dokument s definicí referenčního zařízení.</t>
+    <t>Návrh k týmovému schválení. NFP-02 a NFP-07 čekají na testovací parametry; referenční zařízení pro NFP-17 dosud není určeno. Odkaz na referenční zařízení: https://github.com/Andr3wHere/Fueling_Management_Tool/blob/main/REFERENCE_DEVICE.md</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -312,12 +309,6 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Carlito"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -356,12 +347,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -402,10 +392,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Hypertextový odkaz" xfId="2" builtinId="8"/>
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -617,14 +605,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E45"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="100" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="35.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -799,7 +786,7 @@
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
     </row>
-    <row r="17" spans="1:5" ht="91" customHeight="1">
+    <row r="17" spans="1:4" ht="91" customHeight="1">
       <c r="A17" s="7" t="s">
         <v>34</v>
       </c>
@@ -813,7 +800,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="76" customHeight="1">
+    <row r="18" spans="1:4" ht="76" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>38</v>
       </c>
@@ -827,7 +814,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="26" customHeight="1">
+    <row r="19" spans="1:4" ht="26" customHeight="1">
       <c r="A19" s="9" t="s">
         <v>42</v>
       </c>
@@ -835,7 +822,7 @@
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
-    <row r="20" spans="1:5" ht="61" customHeight="1">
+    <row r="20" spans="1:4" ht="61" customHeight="1">
       <c r="A20" s="7" t="s">
         <v>43</v>
       </c>
@@ -849,7 +836,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="76" customHeight="1">
+    <row r="21" spans="1:4" ht="76" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>47</v>
       </c>
@@ -863,7 +850,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="26" customHeight="1">
+    <row r="22" spans="1:4" ht="26" customHeight="1">
       <c r="A22" s="9" t="s">
         <v>51</v>
       </c>
@@ -871,7 +858,7 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
-    <row r="23" spans="1:5" ht="61" customHeight="1">
+    <row r="23" spans="1:4" ht="61" customHeight="1">
       <c r="A23" s="7" t="s">
         <v>52</v>
       </c>
@@ -885,7 +872,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="76" customHeight="1">
+    <row r="24" spans="1:4" ht="76" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>56</v>
       </c>
@@ -899,7 +886,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="26" customHeight="1">
+    <row r="25" spans="1:4" ht="26" customHeight="1">
       <c r="A25" s="9" t="s">
         <v>59</v>
       </c>
@@ -907,7 +894,7 @@
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
-    <row r="26" spans="1:5" ht="61" customHeight="1">
+    <row r="26" spans="1:4" ht="61" customHeight="1">
       <c r="A26" s="7" t="s">
         <v>60</v>
       </c>
@@ -921,7 +908,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="61" customHeight="1">
+    <row r="27" spans="1:4" ht="61" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
@@ -935,7 +922,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="61" customHeight="1">
+    <row r="28" spans="1:4" ht="61" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>67</v>
       </c>
@@ -949,7 +936,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="76" customHeight="1">
+    <row r="29" spans="1:4" ht="76" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>71</v>
       </c>
@@ -962,17 +949,14 @@
       <c r="D29" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1028,9 +1012,6 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A11:D11"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="E29" r:id="rId1" xr:uid="{1B60EFB6-15CA-4EED-ADA5-9B873EEC2371}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>